<commit_message>
chore(make-36pot): refresh protein-mix-calculator.xlsx from Google Sheets
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/processes/make-36pot/resources/protein-mix-calculator.xlsx
+++ b/docs/processes/make-36pot/resources/protein-mix-calculator.xlsx
@@ -73,17 +73,17 @@
     <t>Protein</t>
   </si>
   <si>
-    <t>Conc
-(ug/mL)</t>
-  </si>
-  <si>
-    <t>Volume (uL)</t>
-  </si>
-  <si>
-    <t>Total Protein (ug)</t>
-  </si>
-  <si>
-    <t>Protein Conc in p-mix (ug/mL)</t>
+    <t>Stock Conc
+(ng/uL)</t>
+  </si>
+  <si>
+    <t>Stock Volume (uL)</t>
+  </si>
+  <si>
+    <t>Available Protein (ug)</t>
+  </si>
+  <si>
+    <t>Protein Conc in p-mix (ng/uL)</t>
   </si>
   <si>
     <t>Protein Req'd (ug)</t>
@@ -200,7 +200,7 @@
     <t>T7RNAP</t>
   </si>
   <si>
-    <t>Total p-mix volume (uL)</t>
+    <t>Total PMix volume (uL)</t>
   </si>
 </sst>
 </file>
@@ -526,9 +526,6 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="13" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="13" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="10" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -557,12 +554,15 @@
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="bottom"/>
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="14" fillId="4" fontId="3" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="14" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
+    <xf borderId="14" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
     <xf borderId="5" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
@@ -586,7 +586,7 @@
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="4" numFmtId="2" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="bottom"/>
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="9" fillId="4" fontId="3" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="10" fillId="0" fontId="3" numFmtId="4" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
@@ -992,7 +992,7 @@
       </c>
       <c r="F10" s="36" t="str">
         <f>if(E10="Yes", CONCATENATE("Concentrate the protein mix (Currently: ",round(I50,1), " uL) using a 3kDa Amicon Filter to ~",(B9-10)," uL"),"")</f>
-        <v>Concentrate the protein mix (Currently: 3619.9 uL) using a 3kDa Amicon Filter to ~230 uL</v>
+        <v>Concentrate the protein mix (Currently: 4429.9 uL) using a 3kDa Amicon Filter to ~230 uL</v>
       </c>
       <c r="G10" s="34"/>
       <c r="H10" s="28"/>
@@ -1027,745 +1027,745 @@
       <c r="C13" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="45" t="s">
+      <c r="D13" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="46" t="s">
+      <c r="E13" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="47"/>
-      <c r="G13" s="48" t="s">
+      <c r="F13" s="46"/>
+      <c r="G13" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="46" t="s">
+      <c r="H13" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="I13" s="46" t="s">
+      <c r="I13" s="45" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="49">
+      <c r="A14" s="48">
         <v>1.0</v>
       </c>
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="51">
+      <c r="C14" s="50">
         <v>911.7086899999999</v>
       </c>
-      <c r="D14" s="52">
+      <c r="D14" s="51">
         <v>756.0</v>
       </c>
-      <c r="E14" s="53">
+      <c r="E14" s="52">
         <f t="shared" ref="E14:E49" si="1">C14*(D14/1000)</f>
         <v>689.2517696</v>
       </c>
-      <c r="F14" s="54"/>
-      <c r="G14" s="55">
-        <v>887.0121130551817</v>
-      </c>
-      <c r="H14" s="53">
+      <c r="F14" s="53"/>
+      <c r="G14" s="54">
+        <v>1086.0</v>
+      </c>
+      <c r="H14" s="52">
         <f t="shared" ref="H14:H49" si="2">G14*($B$9/1000)</f>
-        <v>212.8829071</v>
-      </c>
-      <c r="I14" s="56">
+        <v>260.64</v>
+      </c>
+      <c r="I14" s="55">
         <f t="shared" ref="I14:I49" si="3">H14/(C14/1000)</f>
-        <v>233.4988242</v>
+        <v>285.8807894</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="49">
+      <c r="A15" s="48">
         <v>2.0</v>
       </c>
-      <c r="B15" s="50" t="s">
+      <c r="B15" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="51">
+      <c r="C15" s="50">
         <v>351.56415000000004</v>
       </c>
-      <c r="D15" s="52">
+      <c r="D15" s="51">
         <v>800.0</v>
       </c>
-      <c r="E15" s="53">
+      <c r="E15" s="52">
         <f t="shared" si="1"/>
         <v>281.25132</v>
       </c>
-      <c r="F15" s="57"/>
-      <c r="G15" s="55">
-        <v>24.730820995962315</v>
-      </c>
-      <c r="H15" s="53">
-        <f t="shared" si="2"/>
-        <v>5.935397039</v>
-      </c>
-      <c r="I15" s="56">
-        <f t="shared" si="3"/>
-        <v>16.8828279</v>
+      <c r="F15" s="56"/>
+      <c r="G15" s="54">
+        <v>30.0</v>
+      </c>
+      <c r="H15" s="52">
+        <f t="shared" si="2"/>
+        <v>7.2</v>
+      </c>
+      <c r="I15" s="55">
+        <f t="shared" si="3"/>
+        <v>20.47990388</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="49">
+      <c r="A16" s="48">
         <v>3.0</v>
       </c>
-      <c r="B16" s="50" t="s">
+      <c r="B16" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="51">
+      <c r="C16" s="50">
         <v>480.97093</v>
       </c>
-      <c r="D16" s="52">
+      <c r="D16" s="51">
         <v>420.0</v>
       </c>
-      <c r="E16" s="53">
+      <c r="E16" s="52">
         <f t="shared" si="1"/>
         <v>202.0077906</v>
       </c>
-      <c r="F16" s="54"/>
-      <c r="G16" s="55">
-        <v>278.63391655450874</v>
-      </c>
-      <c r="H16" s="53">
-        <f t="shared" si="2"/>
-        <v>66.87213997</v>
-      </c>
-      <c r="I16" s="56">
-        <f t="shared" si="3"/>
-        <v>139.0357209</v>
+      <c r="F16" s="53"/>
+      <c r="G16" s="54">
+        <v>341.0</v>
+      </c>
+      <c r="H16" s="52">
+        <f t="shared" si="2"/>
+        <v>81.84</v>
+      </c>
+      <c r="I16" s="55">
+        <f t="shared" si="3"/>
+        <v>170.1558138</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="49">
+      <c r="A17" s="48">
         <v>4.0</v>
       </c>
-      <c r="B17" s="50" t="s">
+      <c r="B17" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="51">
+      <c r="C17" s="50">
         <v>811.16708</v>
       </c>
-      <c r="D17" s="52">
+      <c r="D17" s="51">
         <v>800.0</v>
       </c>
-      <c r="E17" s="53">
+      <c r="E17" s="52">
         <f t="shared" si="1"/>
         <v>648.933664</v>
       </c>
-      <c r="F17" s="54"/>
-      <c r="G17" s="55">
-        <v>102.22072678331091</v>
-      </c>
-      <c r="H17" s="53">
-        <f t="shared" si="2"/>
-        <v>24.53297443</v>
-      </c>
-      <c r="I17" s="56">
-        <f t="shared" si="3"/>
-        <v>30.24404593</v>
+      <c r="F17" s="53"/>
+      <c r="G17" s="54">
+        <v>125.0</v>
+      </c>
+      <c r="H17" s="52">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="I17" s="55">
+        <f t="shared" si="3"/>
+        <v>36.98374939</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="49">
+      <c r="A18" s="48">
         <v>5.0</v>
       </c>
-      <c r="B18" s="50" t="s">
+      <c r="B18" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="51">
+      <c r="C18" s="50">
         <v>850.7350700000001</v>
       </c>
-      <c r="D18" s="52">
+      <c r="D18" s="51">
         <v>860.0</v>
       </c>
-      <c r="E18" s="53">
+      <c r="E18" s="52">
         <f t="shared" si="1"/>
         <v>731.6321602</v>
       </c>
-      <c r="F18" s="57"/>
-      <c r="G18" s="55">
-        <v>14.838492597577389</v>
-      </c>
-      <c r="H18" s="53">
-        <f t="shared" si="2"/>
-        <v>3.561238223</v>
-      </c>
-      <c r="I18" s="56">
-        <f t="shared" si="3"/>
-        <v>4.186071962</v>
+      <c r="F18" s="56"/>
+      <c r="G18" s="54">
+        <v>18.0</v>
+      </c>
+      <c r="H18" s="52">
+        <f t="shared" si="2"/>
+        <v>4.32</v>
+      </c>
+      <c r="I18" s="55">
+        <f t="shared" si="3"/>
+        <v>5.07796158</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="49">
+      <c r="A19" s="48">
         <v>6.0</v>
       </c>
-      <c r="B19" s="50" t="s">
+      <c r="B19" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="51">
+      <c r="C19" s="50">
         <v>1472.5888</v>
       </c>
-      <c r="D19" s="52">
+      <c r="D19" s="51">
         <v>800.0</v>
       </c>
-      <c r="E19" s="53">
+      <c r="E19" s="52">
         <f t="shared" si="1"/>
         <v>1178.07104</v>
       </c>
-      <c r="F19" s="57"/>
-      <c r="G19" s="55">
-        <v>47.812920592193805</v>
-      </c>
-      <c r="H19" s="53">
-        <f t="shared" si="2"/>
-        <v>11.47510094</v>
-      </c>
-      <c r="I19" s="56">
-        <f t="shared" si="3"/>
-        <v>7.792467892</v>
+      <c r="F19" s="56"/>
+      <c r="G19" s="54">
+        <v>59.0</v>
+      </c>
+      <c r="H19" s="52">
+        <f t="shared" si="2"/>
+        <v>14.16</v>
+      </c>
+      <c r="I19" s="55">
+        <f t="shared" si="3"/>
+        <v>9.61571893</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="49">
+      <c r="A20" s="48">
         <v>7.0</v>
       </c>
-      <c r="B20" s="50" t="s">
+      <c r="B20" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="51">
+      <c r="C20" s="50">
         <v>3630.85846</v>
       </c>
-      <c r="D20" s="52">
+      <c r="D20" s="51">
         <v>1008.0</v>
       </c>
-      <c r="E20" s="53">
+      <c r="E20" s="52">
         <f t="shared" si="1"/>
         <v>3659.905328</v>
       </c>
-      <c r="F20" s="54"/>
-      <c r="G20" s="55">
-        <v>159.92597577388963</v>
-      </c>
-      <c r="H20" s="53">
-        <f t="shared" si="2"/>
-        <v>38.38223419</v>
-      </c>
-      <c r="I20" s="56">
-        <f t="shared" si="3"/>
-        <v>10.57111827</v>
+      <c r="F20" s="53"/>
+      <c r="G20" s="54">
+        <v>196.0</v>
+      </c>
+      <c r="H20" s="52">
+        <f t="shared" si="2"/>
+        <v>47.04</v>
+      </c>
+      <c r="I20" s="55">
+        <f t="shared" si="3"/>
+        <v>12.95561381</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="49">
+      <c r="A21" s="48">
         <v>8.0</v>
       </c>
-      <c r="B21" s="50" t="s">
+      <c r="B21" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="51">
+      <c r="C21" s="50">
         <v>510.16043</v>
       </c>
-      <c r="D21" s="52">
+      <c r="D21" s="51">
         <v>1180.0</v>
       </c>
-      <c r="E21" s="53">
+      <c r="E21" s="52">
         <f t="shared" si="1"/>
         <v>601.9893074</v>
       </c>
-      <c r="F21" s="54"/>
-      <c r="G21" s="55">
-        <v>122.00538358008075</v>
-      </c>
-      <c r="H21" s="53">
-        <f t="shared" si="2"/>
-        <v>29.28129206</v>
-      </c>
-      <c r="I21" s="56">
-        <f t="shared" si="3"/>
-        <v>57.3962431</v>
+      <c r="F21" s="53"/>
+      <c r="G21" s="54">
+        <v>149.0</v>
+      </c>
+      <c r="H21" s="52">
+        <f t="shared" si="2"/>
+        <v>35.76</v>
+      </c>
+      <c r="I21" s="55">
+        <f t="shared" si="3"/>
+        <v>70.09559718</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="49">
+      <c r="A22" s="48">
         <v>9.0</v>
       </c>
-      <c r="B22" s="50" t="s">
+      <c r="B22" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="51">
+      <c r="C22" s="50">
         <v>1275.55967</v>
       </c>
-      <c r="D22" s="52">
+      <c r="D22" s="51">
         <v>936.0</v>
       </c>
-      <c r="E22" s="53">
+      <c r="E22" s="52">
         <f t="shared" si="1"/>
         <v>1193.923851</v>
       </c>
-      <c r="F22" s="55"/>
-      <c r="G22" s="55">
-        <v>9.892328398384926</v>
-      </c>
-      <c r="H22" s="53">
-        <f t="shared" si="2"/>
-        <v>2.374158816</v>
-      </c>
-      <c r="I22" s="56">
-        <f t="shared" si="3"/>
-        <v>1.861268329</v>
+      <c r="F22" s="57"/>
+      <c r="G22" s="54">
+        <v>12.0</v>
+      </c>
+      <c r="H22" s="52">
+        <f t="shared" si="2"/>
+        <v>2.88</v>
+      </c>
+      <c r="I22" s="55">
+        <f t="shared" si="3"/>
+        <v>2.257832438</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="49">
+      <c r="A23" s="48">
         <v>10.0</v>
       </c>
-      <c r="B23" s="50" t="s">
+      <c r="B23" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="51">
+      <c r="C23" s="50">
         <v>367.13189</v>
       </c>
-      <c r="D23" s="52">
+      <c r="D23" s="51">
         <v>864.0</v>
       </c>
-      <c r="E23" s="53">
+      <c r="E23" s="52">
         <f t="shared" si="1"/>
         <v>317.201953</v>
       </c>
-      <c r="F23" s="54"/>
-      <c r="G23" s="55">
-        <v>507.80619111709285</v>
-      </c>
-      <c r="H23" s="53">
-        <f t="shared" si="2"/>
-        <v>121.8734859</v>
-      </c>
-      <c r="I23" s="56">
-        <f t="shared" si="3"/>
-        <v>331.961045</v>
+      <c r="F23" s="53"/>
+      <c r="G23" s="54">
+        <v>622.0</v>
+      </c>
+      <c r="H23" s="52">
+        <f t="shared" si="2"/>
+        <v>149.28</v>
+      </c>
+      <c r="I23" s="55">
+        <f t="shared" si="3"/>
+        <v>406.6113679</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="49">
+      <c r="A24" s="48">
         <v>11.0</v>
       </c>
-      <c r="B24" s="50" t="s">
+      <c r="B24" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="51">
+      <c r="C24" s="50">
         <v>887.70844</v>
       </c>
-      <c r="D24" s="52">
+      <c r="D24" s="51">
         <v>660.0</v>
       </c>
-      <c r="E24" s="53">
+      <c r="E24" s="52">
         <f t="shared" si="1"/>
         <v>585.8875704</v>
       </c>
-      <c r="F24" s="57"/>
-      <c r="G24" s="55">
-        <v>51.110363391655454</v>
-      </c>
-      <c r="H24" s="53">
-        <f t="shared" si="2"/>
-        <v>12.26648721</v>
-      </c>
-      <c r="I24" s="56">
-        <f t="shared" si="3"/>
-        <v>13.81814869</v>
+      <c r="F24" s="56"/>
+      <c r="G24" s="54">
+        <v>63.0</v>
+      </c>
+      <c r="H24" s="52">
+        <f t="shared" si="2"/>
+        <v>15.12</v>
+      </c>
+      <c r="I24" s="55">
+        <f t="shared" si="3"/>
+        <v>17.0326194</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="49">
+      <c r="A25" s="48">
         <v>12.0</v>
       </c>
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="51">
+      <c r="C25" s="50">
         <v>3767.72478</v>
       </c>
-      <c r="D25" s="52">
+      <c r="D25" s="51">
         <v>950.0</v>
       </c>
-      <c r="E25" s="53">
+      <c r="E25" s="52">
         <f t="shared" si="1"/>
         <v>3579.338541</v>
       </c>
-      <c r="F25" s="57"/>
-      <c r="G25" s="55">
-        <v>80.78734858681023</v>
-      </c>
-      <c r="H25" s="53">
-        <f t="shared" si="2"/>
-        <v>19.38896366</v>
-      </c>
-      <c r="I25" s="56">
-        <f t="shared" si="3"/>
-        <v>5.146066869</v>
+      <c r="F25" s="56"/>
+      <c r="G25" s="54">
+        <v>99.0</v>
+      </c>
+      <c r="H25" s="52">
+        <f t="shared" si="2"/>
+        <v>23.76</v>
+      </c>
+      <c r="I25" s="55">
+        <f t="shared" si="3"/>
+        <v>6.306193097</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="49">
+      <c r="A26" s="48">
         <v>13.0</v>
       </c>
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="51">
+      <c r="C26" s="50">
         <v>185.02844</v>
       </c>
-      <c r="D26" s="52">
+      <c r="D26" s="51">
         <v>708.0</v>
       </c>
-      <c r="E26" s="53">
+      <c r="E26" s="52">
         <f t="shared" si="1"/>
         <v>131.0001355</v>
       </c>
-      <c r="F26" s="57"/>
-      <c r="G26" s="55">
-        <v>29.676985195154778</v>
-      </c>
-      <c r="H26" s="53">
-        <f t="shared" si="2"/>
-        <v>7.122476447</v>
-      </c>
-      <c r="I26" s="56">
-        <f t="shared" si="3"/>
-        <v>38.49395502</v>
+      <c r="F26" s="56"/>
+      <c r="G26" s="54">
+        <v>36.0</v>
+      </c>
+      <c r="H26" s="52">
+        <f t="shared" si="2"/>
+        <v>8.64</v>
+      </c>
+      <c r="I26" s="55">
+        <f t="shared" si="3"/>
+        <v>46.69552421</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="49">
+      <c r="A27" s="48">
         <v>14.0</v>
       </c>
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="C27" s="51">
+      <c r="C27" s="50">
         <v>1088.72338</v>
       </c>
-      <c r="D27" s="52">
+      <c r="D27" s="51">
         <v>864.0</v>
       </c>
-      <c r="E27" s="53">
+      <c r="E27" s="52">
         <f t="shared" si="1"/>
         <v>940.6570003</v>
       </c>
-      <c r="F27" s="54"/>
-      <c r="G27" s="55">
-        <v>215.98250336473754</v>
-      </c>
-      <c r="H27" s="53">
-        <f t="shared" si="2"/>
-        <v>51.83580081</v>
-      </c>
-      <c r="I27" s="56">
-        <f t="shared" si="3"/>
-        <v>47.61154372</v>
+      <c r="F27" s="53"/>
+      <c r="G27" s="54">
+        <v>264.0</v>
+      </c>
+      <c r="H27" s="52">
+        <f t="shared" si="2"/>
+        <v>63.36</v>
+      </c>
+      <c r="I27" s="55">
+        <f t="shared" si="3"/>
+        <v>58.19660087</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="49">
+      <c r="A28" s="48">
         <v>15.0</v>
       </c>
-      <c r="B28" s="50" t="s">
+      <c r="B28" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="51">
+      <c r="C28" s="50">
         <v>314.54503</v>
       </c>
-      <c r="D28" s="52">
+      <c r="D28" s="51">
         <v>936.0</v>
       </c>
-      <c r="E28" s="53">
+      <c r="E28" s="52">
         <f t="shared" si="1"/>
         <v>294.4141481</v>
       </c>
-      <c r="F28" s="54"/>
-      <c r="G28" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H28" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I28" s="56">
-        <f t="shared" si="3"/>
-        <v>96.86489552</v>
+      <c r="F28" s="53"/>
+      <c r="G28" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H28" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I28" s="55">
+        <f t="shared" si="3"/>
+        <v>118.2660556</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="49">
+      <c r="A29" s="48">
         <v>16.0</v>
       </c>
-      <c r="B29" s="50" t="s">
+      <c r="B29" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="C29" s="51">
+      <c r="C29" s="50">
         <v>1718.25073</v>
       </c>
-      <c r="D29" s="52">
+      <c r="D29" s="51">
         <v>954.0</v>
       </c>
-      <c r="E29" s="53">
+      <c r="E29" s="52">
         <f t="shared" si="1"/>
         <v>1639.211196</v>
       </c>
-      <c r="F29" s="57"/>
-      <c r="G29" s="55">
-        <v>24.730820995962315</v>
-      </c>
-      <c r="H29" s="53">
-        <f t="shared" si="2"/>
-        <v>5.935397039</v>
-      </c>
-      <c r="I29" s="56">
-        <f t="shared" si="3"/>
-        <v>3.454325341</v>
+      <c r="F29" s="56"/>
+      <c r="G29" s="54">
+        <v>30.0</v>
+      </c>
+      <c r="H29" s="52">
+        <f t="shared" si="2"/>
+        <v>7.2</v>
+      </c>
+      <c r="I29" s="55">
+        <f t="shared" si="3"/>
+        <v>4.190308128</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="49">
+      <c r="A30" s="48">
         <v>17.0</v>
       </c>
-      <c r="B30" s="50" t="s">
+      <c r="B30" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="51">
+      <c r="C30" s="50">
         <v>600.0</v>
       </c>
-      <c r="D30" s="52">
+      <c r="D30" s="51">
         <v>1080.0</v>
       </c>
-      <c r="E30" s="53">
+      <c r="E30" s="52">
         <f t="shared" si="1"/>
         <v>648</v>
       </c>
-      <c r="F30" s="57"/>
-      <c r="G30" s="55">
-        <v>79.13862718707941</v>
-      </c>
-      <c r="H30" s="53">
-        <f t="shared" si="2"/>
-        <v>18.99327052</v>
-      </c>
-      <c r="I30" s="56">
-        <f t="shared" si="3"/>
-        <v>31.65545087</v>
+      <c r="F30" s="56"/>
+      <c r="G30" s="54">
+        <v>97.0</v>
+      </c>
+      <c r="H30" s="52">
+        <f t="shared" si="2"/>
+        <v>23.28</v>
+      </c>
+      <c r="I30" s="55">
+        <f t="shared" si="3"/>
+        <v>38.8</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="49">
+      <c r="A31" s="48">
         <v>18.0</v>
       </c>
-      <c r="B31" s="50" t="s">
+      <c r="B31" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="C31" s="51">
+      <c r="C31" s="50">
         <v>4345.60133</v>
       </c>
-      <c r="D31" s="52">
+      <c r="D31" s="51">
         <v>914.0</v>
       </c>
-      <c r="E31" s="53">
+      <c r="E31" s="52">
         <f t="shared" si="1"/>
         <v>3971.879616</v>
       </c>
-      <c r="F31" s="57"/>
-      <c r="G31" s="55">
-        <v>79.13862718707941</v>
-      </c>
-      <c r="H31" s="53">
-        <f t="shared" si="2"/>
-        <v>18.99327052</v>
-      </c>
-      <c r="I31" s="56">
-        <f t="shared" si="3"/>
-        <v>4.370688676</v>
+      <c r="F31" s="56"/>
+      <c r="G31" s="54">
+        <v>97.0</v>
+      </c>
+      <c r="H31" s="52">
+        <f t="shared" si="2"/>
+        <v>23.28</v>
+      </c>
+      <c r="I31" s="55">
+        <f t="shared" si="3"/>
+        <v>5.357141218</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="49">
+      <c r="A32" s="48">
         <v>19.0</v>
       </c>
-      <c r="B32" s="50" t="s">
+      <c r="B32" s="49" t="s">
         <v>44</v>
       </c>
-      <c r="C32" s="51">
+      <c r="C32" s="50">
         <v>1454.8522</v>
       </c>
-      <c r="D32" s="52">
+      <c r="D32" s="51">
         <v>1168.0</v>
       </c>
-      <c r="E32" s="53">
+      <c r="E32" s="52">
         <f t="shared" si="1"/>
         <v>1699.26737</v>
       </c>
-      <c r="F32" s="55"/>
-      <c r="G32" s="55">
-        <v>8.243606998654105</v>
-      </c>
-      <c r="H32" s="53">
-        <f t="shared" si="2"/>
-        <v>1.97846568</v>
-      </c>
-      <c r="I32" s="56">
-        <f t="shared" si="3"/>
-        <v>1.359908367</v>
+      <c r="F32" s="57"/>
+      <c r="G32" s="54">
+        <v>10.0</v>
+      </c>
+      <c r="H32" s="52">
+        <f t="shared" si="2"/>
+        <v>2.4</v>
+      </c>
+      <c r="I32" s="55">
+        <f t="shared" si="3"/>
+        <v>1.649652109</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="49">
+      <c r="A33" s="48">
         <v>20.0</v>
       </c>
-      <c r="B33" s="50" t="s">
+      <c r="B33" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="C33" s="51">
+      <c r="C33" s="50">
         <v>619.34709</v>
       </c>
-      <c r="D33" s="52">
+      <c r="D33" s="51">
         <v>752.0</v>
       </c>
-      <c r="E33" s="53">
+      <c r="E33" s="52">
         <f t="shared" si="1"/>
         <v>465.7490117</v>
       </c>
-      <c r="F33" s="57"/>
-      <c r="G33" s="55">
-        <v>23.082099596231494</v>
-      </c>
-      <c r="H33" s="53">
-        <f t="shared" si="2"/>
-        <v>5.539703903</v>
-      </c>
-      <c r="I33" s="56">
-        <f t="shared" si="3"/>
-        <v>8.944425497</v>
+      <c r="F33" s="56"/>
+      <c r="G33" s="54">
+        <v>28.0</v>
+      </c>
+      <c r="H33" s="52">
+        <f t="shared" si="2"/>
+        <v>6.72</v>
+      </c>
+      <c r="I33" s="55">
+        <f t="shared" si="3"/>
+        <v>10.85013575</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="49">
+      <c r="A34" s="48">
         <v>21.0</v>
       </c>
       <c r="B34" s="58" t="s">
         <v>46</v>
       </c>
-      <c r="C34" s="51">
+      <c r="C34" s="50">
         <v>758.2683099999999</v>
       </c>
-      <c r="D34" s="52">
+      <c r="D34" s="51">
         <v>568.0</v>
       </c>
-      <c r="E34" s="53">
+      <c r="E34" s="52">
         <f t="shared" si="1"/>
         <v>430.6964001</v>
       </c>
-      <c r="F34" s="54"/>
-      <c r="G34" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H34" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I34" s="56">
-        <f t="shared" si="3"/>
-        <v>40.18151763</v>
+      <c r="F34" s="53"/>
+      <c r="G34" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H34" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I34" s="55">
+        <f t="shared" si="3"/>
+        <v>49.05915163</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="49">
+      <c r="A35" s="48">
         <v>22.0</v>
       </c>
       <c r="B35" s="58" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="51">
+      <c r="C35" s="50">
         <v>450.0</v>
       </c>
-      <c r="D35" s="52">
+      <c r="D35" s="51">
         <v>1100.0</v>
       </c>
-      <c r="E35" s="53">
+      <c r="E35" s="52">
         <f t="shared" si="1"/>
         <v>495</v>
       </c>
-      <c r="F35" s="54"/>
-      <c r="G35" s="55">
-        <v>507.80619111709285</v>
-      </c>
-      <c r="H35" s="53">
-        <f t="shared" si="2"/>
-        <v>121.8734859</v>
-      </c>
-      <c r="I35" s="56">
-        <f t="shared" si="3"/>
-        <v>270.8299686</v>
+      <c r="F35" s="53"/>
+      <c r="G35" s="54">
+        <v>622.0</v>
+      </c>
+      <c r="H35" s="52">
+        <f t="shared" si="2"/>
+        <v>149.28</v>
+      </c>
+      <c r="I35" s="55">
+        <f t="shared" si="3"/>
+        <v>331.7333333</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="49">
+      <c r="A36" s="48">
         <v>23.0</v>
       </c>
       <c r="B36" s="58" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="51">
+      <c r="C36" s="50">
         <v>953.0176799999999</v>
       </c>
-      <c r="D36" s="52">
+      <c r="D36" s="51">
         <v>558.0</v>
       </c>
-      <c r="E36" s="53">
+      <c r="E36" s="52">
         <f t="shared" si="1"/>
         <v>531.7838654</v>
       </c>
-      <c r="F36" s="54"/>
-      <c r="G36" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H36" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I36" s="56">
-        <f t="shared" si="3"/>
-        <v>31.97041577</v>
+      <c r="F36" s="53"/>
+      <c r="G36" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H36" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I36" s="55">
+        <f t="shared" si="3"/>
+        <v>39.03390334</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="49">
+      <c r="A37" s="48">
         <v>24.0</v>
       </c>
       <c r="B37" s="58" t="s">
         <v>49</v>
       </c>
-      <c r="C37" s="51">
+      <c r="C37" s="50">
         <v>1590.0</v>
       </c>
-      <c r="D37" s="52">
+      <c r="D37" s="51">
         <v>640.0</v>
       </c>
-      <c r="E37" s="53">
+      <c r="E37" s="52">
         <f t="shared" si="1"/>
         <v>1017.6</v>
       </c>
-      <c r="F37" s="54"/>
-      <c r="G37" s="55">
-        <v>634.757738896366</v>
-      </c>
-      <c r="H37" s="53">
-        <f t="shared" si="2"/>
-        <v>152.3418573</v>
-      </c>
-      <c r="I37" s="56">
-        <f t="shared" si="3"/>
-        <v>95.81248889</v>
+      <c r="F37" s="53"/>
+      <c r="G37" s="54">
+        <v>777.0</v>
+      </c>
+      <c r="H37" s="52">
+        <f t="shared" si="2"/>
+        <v>186.48</v>
+      </c>
+      <c r="I37" s="55">
+        <f t="shared" si="3"/>
+        <v>117.2830189</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="49">
+      <c r="A38" s="48">
         <v>25.0</v>
       </c>
       <c r="B38" s="58" t="s">
@@ -1774,28 +1774,28 @@
       <c r="C38" s="59">
         <v>940.0</v>
       </c>
-      <c r="D38" s="52">
+      <c r="D38" s="51">
         <v>2620.0</v>
       </c>
-      <c r="E38" s="53">
+      <c r="E38" s="52">
         <f t="shared" si="1"/>
         <v>2462.8</v>
       </c>
-      <c r="F38" s="54"/>
-      <c r="G38" s="55">
-        <v>6340.982503364738</v>
-      </c>
-      <c r="H38" s="53">
-        <f t="shared" si="2"/>
-        <v>1521.835801</v>
-      </c>
-      <c r="I38" s="56">
-        <f t="shared" si="3"/>
-        <v>1618.974256</v>
+      <c r="F38" s="53"/>
+      <c r="G38" s="54">
+        <v>7764.0</v>
+      </c>
+      <c r="H38" s="52">
+        <f t="shared" si="2"/>
+        <v>1863.36</v>
+      </c>
+      <c r="I38" s="55">
+        <f t="shared" si="3"/>
+        <v>1982.297872</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="49">
+      <c r="A39" s="48">
         <v>26.0</v>
       </c>
       <c r="B39" s="58" t="s">
@@ -1804,294 +1804,294 @@
       <c r="C39" s="59">
         <v>1000.0</v>
       </c>
-      <c r="D39" s="52">
+      <c r="D39" s="51">
         <v>900.0</v>
       </c>
-      <c r="E39" s="53">
+      <c r="E39" s="52">
         <f t="shared" si="1"/>
         <v>900</v>
       </c>
-      <c r="F39" s="54"/>
-      <c r="G39" s="55">
-        <v>634.757738896366</v>
-      </c>
-      <c r="H39" s="53">
-        <f t="shared" si="2"/>
-        <v>152.3418573</v>
-      </c>
-      <c r="I39" s="56">
-        <f t="shared" si="3"/>
-        <v>152.3418573</v>
+      <c r="F39" s="53"/>
+      <c r="G39" s="54">
+        <v>777.0</v>
+      </c>
+      <c r="H39" s="52">
+        <f t="shared" si="2"/>
+        <v>186.48</v>
+      </c>
+      <c r="I39" s="55">
+        <f t="shared" si="3"/>
+        <v>186.48</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="49">
+      <c r="A40" s="48">
         <v>27.0</v>
       </c>
       <c r="B40" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="51">
+      <c r="C40" s="50">
         <v>473.65126000000004</v>
       </c>
-      <c r="D40" s="52">
+      <c r="D40" s="51">
         <v>494.0</v>
       </c>
-      <c r="E40" s="53">
+      <c r="E40" s="52">
         <f t="shared" si="1"/>
         <v>233.9837224</v>
       </c>
-      <c r="F40" s="54"/>
-      <c r="G40" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H40" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I40" s="56">
-        <f t="shared" si="3"/>
-        <v>64.32659224</v>
+      <c r="F40" s="53"/>
+      <c r="G40" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H40" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I40" s="55">
+        <f t="shared" si="3"/>
+        <v>78.53879667</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="49">
+      <c r="A41" s="48">
         <v>28.0</v>
       </c>
       <c r="B41" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="51">
+      <c r="C41" s="50">
         <v>807.57119</v>
       </c>
-      <c r="D41" s="52">
+      <c r="D41" s="51">
         <v>482.0</v>
       </c>
-      <c r="E41" s="53">
+      <c r="E41" s="52">
         <f t="shared" si="1"/>
         <v>389.2493136</v>
       </c>
-      <c r="F41" s="54"/>
-      <c r="G41" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H41" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I41" s="56">
-        <f t="shared" si="3"/>
-        <v>37.7284032</v>
+      <c r="F41" s="53"/>
+      <c r="G41" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H41" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I41" s="55">
+        <f t="shared" si="3"/>
+        <v>46.0640504</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="49">
+      <c r="A42" s="48">
         <v>29.0</v>
       </c>
       <c r="B42" s="58" t="s">
         <v>54</v>
       </c>
-      <c r="C42" s="51">
+      <c r="C42" s="50">
         <v>846.5157399999999</v>
       </c>
-      <c r="D42" s="52">
+      <c r="D42" s="51">
         <v>488.0</v>
       </c>
-      <c r="E42" s="53">
+      <c r="E42" s="52">
         <f t="shared" si="1"/>
         <v>413.0996811</v>
       </c>
-      <c r="F42" s="54"/>
-      <c r="G42" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H42" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I42" s="56">
-        <f t="shared" si="3"/>
-        <v>35.99268156</v>
+      <c r="F42" s="53"/>
+      <c r="G42" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H42" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I42" s="55">
+        <f t="shared" si="3"/>
+        <v>43.94484147</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="49">
+      <c r="A43" s="48">
         <v>30.0</v>
       </c>
       <c r="B43" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="51">
+      <c r="C43" s="50">
         <v>1463.09053</v>
       </c>
-      <c r="D43" s="52">
+      <c r="D43" s="51">
         <v>532.0</v>
       </c>
-      <c r="E43" s="53">
+      <c r="E43" s="52">
         <f t="shared" si="1"/>
         <v>778.364162</v>
       </c>
-      <c r="F43" s="54"/>
-      <c r="G43" s="55">
-        <v>126.95154777927321</v>
-      </c>
-      <c r="H43" s="53">
-        <f t="shared" si="2"/>
-        <v>30.46837147</v>
-      </c>
-      <c r="I43" s="56">
-        <f t="shared" si="3"/>
-        <v>20.8246659</v>
+      <c r="F43" s="53"/>
+      <c r="G43" s="54">
+        <v>155.0</v>
+      </c>
+      <c r="H43" s="52">
+        <f t="shared" si="2"/>
+        <v>37.2</v>
+      </c>
+      <c r="I43" s="55">
+        <f t="shared" si="3"/>
+        <v>25.42563104</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="49">
+      <c r="A44" s="48">
         <v>31.0</v>
       </c>
       <c r="B44" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="C44" s="51">
+      <c r="C44" s="50">
         <v>3608.8898999999997</v>
       </c>
-      <c r="D44" s="52">
+      <c r="D44" s="51">
         <v>520.0</v>
       </c>
-      <c r="E44" s="53">
+      <c r="E44" s="52">
         <f t="shared" si="1"/>
         <v>1876.622748</v>
       </c>
-      <c r="F44" s="54"/>
-      <c r="G44" s="55">
-        <v>253.90309555854643</v>
-      </c>
-      <c r="H44" s="53">
-        <f t="shared" si="2"/>
-        <v>60.93674293</v>
-      </c>
-      <c r="I44" s="56">
-        <f t="shared" si="3"/>
-        <v>16.8851765</v>
+      <c r="F44" s="53"/>
+      <c r="G44" s="54">
+        <v>311.0</v>
+      </c>
+      <c r="H44" s="52">
+        <f t="shared" si="2"/>
+        <v>74.64</v>
+      </c>
+      <c r="I44" s="55">
+        <f t="shared" si="3"/>
+        <v>20.68226022</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="49">
+      <c r="A45" s="48">
         <v>32.0</v>
       </c>
       <c r="B45" s="58" t="s">
         <v>57</v>
       </c>
-      <c r="C45" s="51">
+      <c r="C45" s="50">
         <v>504.29616</v>
       </c>
-      <c r="D45" s="52">
+      <c r="D45" s="51">
         <v>534.0</v>
       </c>
-      <c r="E45" s="53">
+      <c r="E45" s="52">
         <f t="shared" si="1"/>
         <v>269.2941494</v>
       </c>
-      <c r="F45" s="57"/>
-      <c r="G45" s="55">
-        <v>51.110363391655454</v>
-      </c>
-      <c r="H45" s="53">
-        <f t="shared" si="2"/>
-        <v>12.26648721</v>
-      </c>
-      <c r="I45" s="56">
-        <f t="shared" si="3"/>
-        <v>24.32397505</v>
+      <c r="F45" s="56"/>
+      <c r="G45" s="54">
+        <v>63.0</v>
+      </c>
+      <c r="H45" s="52">
+        <f t="shared" si="2"/>
+        <v>15.12</v>
+      </c>
+      <c r="I45" s="55">
+        <f t="shared" si="3"/>
+        <v>29.98238178</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="49">
+      <c r="A46" s="48">
         <v>33.0</v>
       </c>
-      <c r="B46" s="50" t="s">
+      <c r="B46" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="C46" s="51">
+      <c r="C46" s="50">
         <v>1266.29284</v>
       </c>
-      <c r="D46" s="52">
+      <c r="D46" s="51">
         <v>466.0</v>
       </c>
-      <c r="E46" s="53">
+      <c r="E46" s="52">
         <f t="shared" si="1"/>
         <v>590.0924634</v>
       </c>
-      <c r="F46" s="57"/>
-      <c r="G46" s="55">
-        <v>37.920592193808886</v>
-      </c>
-      <c r="H46" s="53">
-        <f t="shared" si="2"/>
-        <v>9.100942127</v>
-      </c>
-      <c r="I46" s="56">
-        <f t="shared" si="3"/>
-        <v>7.187075405</v>
+      <c r="F46" s="56"/>
+      <c r="G46" s="54">
+        <v>46.0</v>
+      </c>
+      <c r="H46" s="52">
+        <f t="shared" si="2"/>
+        <v>11.04</v>
+      </c>
+      <c r="I46" s="55">
+        <f t="shared" si="3"/>
+        <v>8.718362492</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="49">
+      <c r="A47" s="48">
         <v>34.0</v>
       </c>
       <c r="B47" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="C47" s="51">
+      <c r="C47" s="50">
         <v>362.56352</v>
       </c>
-      <c r="D47" s="52">
+      <c r="D47" s="51">
         <v>620.0</v>
       </c>
-      <c r="E47" s="53">
+      <c r="E47" s="52">
         <f t="shared" si="1"/>
         <v>224.7893824</v>
       </c>
-      <c r="F47" s="57"/>
-      <c r="G47" s="55">
-        <v>13.189771197846568</v>
-      </c>
-      <c r="H47" s="53">
-        <f t="shared" si="2"/>
-        <v>3.165545087</v>
-      </c>
-      <c r="I47" s="56">
-        <f t="shared" si="3"/>
-        <v>8.731008259</v>
+      <c r="F47" s="56"/>
+      <c r="G47" s="54">
+        <v>16.0</v>
+      </c>
+      <c r="H47" s="52">
+        <f t="shared" si="2"/>
+        <v>3.84</v>
+      </c>
+      <c r="I47" s="55">
+        <f t="shared" si="3"/>
+        <v>10.59124757</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="49">
+      <c r="A48" s="48">
         <v>35.0</v>
       </c>
       <c r="B48" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="51">
+      <c r="C48" s="50">
         <v>877.1606400000001</v>
       </c>
-      <c r="D48" s="52">
+      <c r="D48" s="51">
         <v>1800.0</v>
       </c>
-      <c r="E48" s="53">
+      <c r="E48" s="52">
         <f t="shared" si="1"/>
         <v>1578.889152</v>
       </c>
-      <c r="F48" s="57"/>
-      <c r="G48" s="55">
-        <v>13.189771197846568</v>
-      </c>
-      <c r="H48" s="53">
-        <f t="shared" si="2"/>
-        <v>3.165545087</v>
-      </c>
-      <c r="I48" s="56">
-        <f t="shared" si="3"/>
-        <v>3.60885446</v>
+      <c r="F48" s="56"/>
+      <c r="G48" s="54">
+        <v>16.0</v>
+      </c>
+      <c r="H48" s="52">
+        <f t="shared" si="2"/>
+        <v>3.84</v>
+      </c>
+      <c r="I48" s="55">
+        <f t="shared" si="3"/>
+        <v>4.37776141</v>
       </c>
     </row>
     <row r="49">
@@ -2113,15 +2113,15 @@
       </c>
       <c r="F49" s="65"/>
       <c r="G49" s="66">
-        <v>126.95154777927321</v>
+        <v>155.0</v>
       </c>
       <c r="H49" s="64">
         <f t="shared" si="2"/>
-        <v>30.46837147</v>
+        <v>37.2</v>
       </c>
       <c r="I49" s="67">
         <f t="shared" si="3"/>
-        <v>105.0633499</v>
+        <v>128.2758621</v>
       </c>
     </row>
     <row r="50">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="I50" s="68">
         <f>SUM(I14:I49)</f>
-        <v>3619.931329</v>
+        <v>4429.947053</v>
       </c>
     </row>
   </sheetData>

</xml_diff>